<commit_message>
fix(import): restore ID column first for NocoBase subscription_branding template
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/import/nocobase-subscription_branding-RU-titles.xlsx
+++ b/import/nocobase-subscription_branding-RU-titles.xlsx
@@ -413,50 +413,55 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>Заголовок подписки</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>URL поддержки</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>URL профиля</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Объявление</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Активен</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>VL</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>https://t.me/VL_VPNbot</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr"/>
-      <c r="E2" t="b">
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>